<commit_message>
Fix agreement edit re-generation and Excel log update
</commit_message>
<xml_diff>
--- a/backend/data/agreements_log.xlsx
+++ b/backend/data/agreements_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:S11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -510,6 +510,956 @@
       <c r="S1" t="inlineStr">
         <is>
           <t>msd_signature_path</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>c3d12f06-63b1-4101-88a1-3a703eb40ce5</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-08-19T00:17:07.725532</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>abc@gmail.com</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Haryana</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>C:\Users\Admin\Desktop\agreement poc\backend\data\signatures\d3047923-479f-4300-94f2-ecd31fce3f8e\customer_customer_signature.png</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>C:\Users\Admin\Desktop\agreement poc\backend\data\signatures\d3047923-479f-4300-94f2-ecd31fce3f8e\msd_msd_signature.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>072a12a9-2a4e-45e7-8935-64c583ddf917</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-08-19T00:19:31.948465</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals Enterprise Ltd</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Greams Lane, 1, Greams Rd, Thousand Lights, Chennai, Tamil Nadu 600006</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Dr. Rajesh Sharma</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Head of Medical Procurement</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>rajesh.sharma@apollohospitals.com</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>+91-9876543210</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2025-04-01</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Advanced Diagnostic Imaging Scanner Model X</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>SN-APOLLO-2025-9988</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>7500000</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Device Purchase Agreement</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>C:\Users\Admin\Desktop\agreement poc\backend\data\signatures\3fa62241-ac40-47bf-a23b-32f41ae6b4e9\customer_cust_sig.png</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>C:\Users\Admin\Desktop\agreement poc\backend\data\signatures\3fa62241-ac40-47bf-a23b-32f41ae6b4e9\msd_comp_sig.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>77a30dca-8e1f-48a1-beae-2a425137e4f9</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-08-19T00:20:33.581994</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>abc@gmail.com</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Haryana</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>C:\Users\Admin\Desktop\agreement poc\backend\data\signatures\7b6d2247-d8cc-4366-b99d-77ec84c09a4f\customer_customer_signature.png</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>C:\Users\Admin\Desktop\agreement poc\backend\data\signatures\7b6d2247-d8cc-4366-b99d-77ec84c09a4f\msd_msd_signature.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>80f15532-992f-435d-af89-48efdebca786</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-08-19T00:27:29.123788</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>abc@gmail.com</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Haryana</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>C:\Users\Admin\Desktop\agreement poc\backend\data\signatures\2454454a-81ed-4976-a2c5-7e3bdd0d0719\customer_customer_signature.png</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>C:\Users\Admin\Desktop\agreement poc\backend\data\signatures\2454454a-81ed-4976-a2c5-7e3bdd0d0719\msd_msd_signature.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>49bc7e92-74df-4771-a443-7ae1bb0b32b5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-08-19T00:31:38.890795</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>abc@gmail.com</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Haryana</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>C:\Users\Admin\Desktop\agreement poc\backend\data\signatures\49eaef11-359f-494d-98e4-8009c15ac45b\customer_customer_signature.png</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>C:\Users\Admin\Desktop\agreement poc\backend\data\signatures\49eaef11-359f-494d-98e4-8009c15ac45b\msd_msd_signature.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>3eb9cab8-ce07-4a6f-a64f-67d678b32198</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-08-19T00:33:14.946471</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>abc@gmail.com</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Haryana</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>999904</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>C:\Users\Admin\Desktop\agreement poc\backend\data\signatures\4cf2cffc-5ddc-47e2-be88-59c091c06406\customer_customer_signature.png</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>C:\Users\Admin\Desktop\agreement poc\backend\data\signatures\4cf2cffc-5ddc-47e2-be88-59c091c06406\msd_msd_signature.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>93921c25-30c0-493f-9bcf-7a134923538f</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-08-19T00:46:20.247073</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals Enterprise Ltd</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Greams Lane, 1, Greams Rd, Thousand Lights, Chennai, Tamil Nadu 600006</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Dr. Rajesh Sharma</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Head of Medical Procurement</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>rajesh.sharma@apollohospitals.com</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>+91-9876543210</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2025-04-01</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Advanced Diagnostic Imaging Scanner Model X</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>SN-APOLLO-2025-9988</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>7500000</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Device Purchase Agreement</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>C:\Users\Admin\Desktop\agreement poc\backend\data\signatures\93921c25-30c0-493f-9bcf-7a134923538f\customer_cust_sig.png</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>C:\Users\Admin\Desktop\agreement poc\backend\data\signatures\93921c25-30c0-493f-9bcf-7a134923538f\msd_comp_sig.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>19c516b4-1a29-4b43-83a2-63049719dc73</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-08-19T00:47:49.013900</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals Enterprise Ltd</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Greams Lane, 1, Greams Rd, Thousand Lights, Chennai, Tamil Nadu 600006</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Dr. Rajesh Sharma</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Head of Medical Procurement</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>rajesh.sharma@apollohospitals.com</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>+91-9876543210</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2025-04-01</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Advanced Diagnostic Imaging Scanner Model X</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>SN-APOLLO-2025-9988</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>7500000</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Device Purchase Agreement</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>C:\Users\Admin\Desktop\agreement poc\backend\data\signatures\19c516b4-1a29-4b43-83a2-63049719dc73\customer_cust_sig.png</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>C:\Users\Admin\Desktop\agreement poc\backend\data\signatures\19c516b4-1a29-4b43-83a2-63049719dc73\msd_comp_sig.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>cedaca1d-3448-4423-ab3d-d8a62c354390</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-08-19T00:49:17.840873</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>abc@gmail.com</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Haryana</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>100000000000</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>C:\Users\Admin\Desktop\agreement poc\backend\data\signatures\cedaca1d-3448-4423-ab3d-d8a62c354390\customer_customer_signature.png</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>C:\Users\Admin\Desktop\agreement poc\backend\data\signatures\cedaca1d-3448-4423-ab3d-d8a62c354390\msd_msd_signature.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>5b3a283d-2551-4554-891d-fdc3b8714a4c</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-08-19T00:54:39.774911</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>abc@gmail.com</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Haryana</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>10000000000000</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>C:\Users\Admin\Desktop\agreement poc\backend\data\signatures\5b3a283d-2551-4554-891d-fdc3b8714a4c\customer_customer_signature.png</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>C:\Users\Admin\Desktop\agreement poc\backend\data\signatures\5b3a283d-2551-4554-891d-fdc3b8714a4c\msd_msd_signature.png</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add setup scripts, document templates, and update launcher with environment path configuration
</commit_message>
<xml_diff>
--- a/backend/data/agreements_log.xlsx
+++ b/backend/data/agreements_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S11"/>
+  <dimension ref="A1:S12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1460,6 +1460,101 @@
       <c r="S11" t="inlineStr">
         <is>
           <t>C:\Users\Admin\Desktop\agreement poc\backend\data\signatures\5b3a283d-2551-4554-891d-fdc3b8714a4c\msd_msd_signature.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>be16cc4d-cd97-46c9-a3ca-902b931cceae</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-08-21T17:04:11.100219</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Ambar</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>lalalala</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Abhishek</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>amb@gmail.com</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>5484564892</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>credence</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>789</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Punjab</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>500000</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Device Purchase Agreement</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>C:\Users\ambar\OneDrive\Desktop\Website\backend\data\signatures\be16cc4d-cd97-46c9-a3ca-902b931cceae\customer_customer_signature.png</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>C:\Users\ambar\OneDrive\Desktop\Website\backend\data\signatures\be16cc4d-cd97-46c9-a3ca-902b931cceae\msd_msd_signature.png</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement comprehensive agreement generation system with date and folder validation modules
</commit_message>
<xml_diff>
--- a/backend/data/agreements_log.xlsx
+++ b/backend/data/agreements_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S12"/>
+  <dimension ref="A1:S14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1555,6 +1555,196 @@
       <c r="S12" t="inlineStr">
         <is>
           <t>C:\Users\ambar\OneDrive\Desktop\Website\backend\data\signatures\be16cc4d-cd97-46c9-a3ca-902b931cceae\msd_msd_signature.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>5bc961e7-5c84-48bc-b1a1-d64ff4fff581</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-08-21T17:38:28.079381</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ambar</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>nyati county, undri, pune</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>abhishek</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>manager</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>abc@gmail.com</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>5484564892</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>credence</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Punjab</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>2</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>msd</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>C:\Users\ambar\OneDrive\Desktop\Website\backend\data\signatures\5bc961e7-5c84-48bc-b1a1-d64ff4fff581\customer_customer_signature.png</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>C:\Users\ambar\OneDrive\Desktop\Website\backend\data\signatures\5bc961e7-5c84-48bc-b1a1-d64ff4fff581\msd_msd_signature.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ded8ce5a-08a5-4feb-bf0c-a8610581bdfd</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-08-21T17:38:35.924768</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ambar</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>nyati county, undri, pune</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>abhishek</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>manager</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>abc@gmail.com</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>5484564892</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>credence</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Punjab</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>2</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Device Purchase Agreement</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>CANCELLED</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>C:\Users\ambar\OneDrive\Desktop\Website\backend\data\signatures\ded8ce5a-08a5-4feb-bf0c-a8610581bdfd\customer_customer_signature.png</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>C:\Users\ambar\OneDrive\Desktop\Website\backend\data\signatures\ded8ce5a-08a5-4feb-bf0c-a8610581bdfd\msd_msd_signature.png</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add standard agreement document templates and initialize the agreements log file
</commit_message>
<xml_diff>
--- a/backend/data/agreements_log.xlsx
+++ b/backend/data/agreements_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S14"/>
+  <dimension ref="A1:S17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1745,6 +1745,291 @@
       <c r="S14" t="inlineStr">
         <is>
           <t>C:\Users\ambar\OneDrive\Desktop\Website\backend\data\signatures\ded8ce5a-08a5-4feb-bf0c-a8610581bdfd\msd_msd_signature.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ef0d4559-2eb7-4b5a-aae2-fed26dc28a91</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-08-24T20:51:24.833657</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ambar</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>lalalala</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>abhishek</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>manager</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>abc@gmail.com</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>5484564892</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>credence</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Punjab</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>2</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Device Purchase Agreement</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>C:\Users\ambar\OneDrive\Desktop\Website\backend\data\signatures\ef0d4559-2eb7-4b5a-aae2-fed26dc28a91\customer_customer_signature.png</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>C:\Users\ambar\OneDrive\Desktop\Website\backend\data\signatures\ef0d4559-2eb7-4b5a-aae2-fed26dc28a91\msd_msd_signature.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>8638c622-1288-40e3-91b6-9ed9627544b3</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-08-24T20:55:15.963103</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals Enterprise Ltd</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Greams Lane, 1, Greams Rd, Thousand Lights, Chennai, Tamil Nadu 600006</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Dr. Rajesh Sharma (Updated)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Head of Medical Procurement</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>rajesh.sharma@apollohospitals.com</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>+91-9876543210</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2025-04-01</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Advanced Diagnostic Imaging Scanner Model X</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>SN-APOLLO-2025-9988</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>8500000</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Device Purchase Agreement</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>C:\Users\ambar\OneDrive\Desktop\Website\backend\data\signatures\8638c622-1288-40e3-91b6-9ed9627544b3\customer_cust_sig.png</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>C:\Users\ambar\OneDrive\Desktop\Website\backend\data\signatures\8638c622-1288-40e3-91b6-9ed9627544b3\msd_comp_sig.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>56c72bba-de9f-4584-9303-252faa0181b7</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-08-24T20:57:38.034925</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals Enterprise Ltd</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Greams Lane, 1, Greams Rd, Thousand Lights, Chennai, Tamil Nadu 600006</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Dr. Rajesh Sharma (Updated)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Head of Medical Procurement</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>rajesh.sharma@apollohospitals.com</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>+91-9876543210</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2025-04-01</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Advanced Diagnostic Imaging Scanner Model X</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>SN-APOLLO-2025-9988</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>8500000</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Device Purchase Agreement</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>C:\Users\ambar\OneDrive\Desktop\Website\backend\data\signatures\56c72bba-de9f-4584-9303-252faa0181b7\customer_cust_sig.png</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>C:\Users\ambar\OneDrive\Desktop\Website\backend\data\signatures\56c72bba-de9f-4584-9303-252faa0181b7\msd_comp_sig.png</t>
         </is>
       </c>
     </row>

</xml_diff>